<commit_message>
fix: GlobalSpinner no bloquea SweetAlert2 ni Colorbox popups
- Agrega guardia Swal.isVisible() en GlobalSpinner.show() para evitar
  que el spinner aparezca encima de un diálogo SweetAlert activo
- Agrega GlobalSpinner.showForced() para usar después del cierre de Swal
- Handler de links ahora verifica e.defaultPrevented antes de activar
  el spinner, lo que excluye automáticamente jQuery Colorbox, Bootstrap
  modals y cualquier handler que ya haya llamado preventDefault
- Excluye explícitamente clases de Colorbox (.popupventana, .popupcomentario,
  .popuprevisar) y triggers de Bootstrap (data-bs-toggle, data-toggle)
- Botones .sweet-* ahora muestran el spinner via willClose del Swal de
  éxito, garantizando que Swal ya cerró cuando el spinner entra
- attachSwalConfirmToForms usa el mismo patrón willClose + form.submit()
  ya que form.submit() nativo no dispara el evento submit

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/seeders/Usuarios.xlsx
+++ b/database/seeders/Usuarios.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20415"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\servidor\Seguimiento\database\seeders\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11DA5458-EA69-4AED-A37E-A591862A020E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B79C055B-1F99-4D59-B943-EDD0E4B56B1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{927018C0-BB9F-433A-9F90-4096039434DC}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="150">
   <si>
     <t>nombre</t>
   </si>
@@ -475,34 +475,13 @@
   </si>
   <si>
     <t>maricela.love.07@gmail.com</t>
-  </si>
-  <si>
-    <t>Jorge Angel Becerril Gonzalez</t>
-  </si>
-  <si>
-    <t>desarrollador.f@osfem.gob.mx</t>
-  </si>
-  <si>
-    <t>Staff Juridico</t>
-  </si>
-  <si>
-    <t>STAFF</t>
-  </si>
-  <si>
-    <t>CA</t>
-  </si>
-  <si>
-    <t>Consultor Administrativo</t>
-  </si>
-  <si>
-    <t>consultoradmin@osfem.gob.mx</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -549,15 +528,8 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -612,13 +584,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -641,24 +608,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -756,24 +711,12 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
-    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -798,9 +741,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -838,7 +781,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -944,7 +887,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1086,7 +1029,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1094,7 +1037,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{850591BD-AB77-48DF-A9A3-0C3060FEC0A7}">
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.85546875" customWidth="1"/>
@@ -2439,7 +2382,7 @@
       <c r="A59" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B59" s="42" t="s">
+      <c r="B59" s="37" t="s">
         <v>123</v>
       </c>
       <c r="C59" s="24" t="s">
@@ -2663,52 +2606,6 @@
       </c>
       <c r="G68" s="29">
         <v>1632</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" s="37" t="s">
-        <v>150</v>
-      </c>
-      <c r="B69" s="38" t="s">
-        <v>151</v>
-      </c>
-      <c r="C69" s="39" t="s">
-        <v>152</v>
-      </c>
-      <c r="D69" s="41">
-        <v>122100</v>
-      </c>
-      <c r="E69" s="40" t="s">
-        <v>152</v>
-      </c>
-      <c r="F69" s="40" t="s">
-        <v>153</v>
-      </c>
-      <c r="G69" s="40">
-        <v>1633</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="37" t="s">
-        <v>155</v>
-      </c>
-      <c r="B70" s="38" t="s">
-        <v>156</v>
-      </c>
-      <c r="C70" s="39" t="s">
-        <v>155</v>
-      </c>
-      <c r="D70" s="41">
-        <v>122000</v>
-      </c>
-      <c r="E70" s="40" t="s">
-        <v>155</v>
-      </c>
-      <c r="F70" s="40" t="s">
-        <v>154</v>
-      </c>
-      <c r="G70" s="40">
-        <v>1634</v>
       </c>
     </row>
   </sheetData>
@@ -2776,9 +2673,8 @@
     <hyperlink ref="B23" r:id="rId61" xr:uid="{A1FAC0C9-F87F-4095-AB0F-7DA09DCED449}"/>
     <hyperlink ref="B35" r:id="rId62" xr:uid="{110808D9-04E6-414C-82E6-5570FD935054}"/>
     <hyperlink ref="B47" r:id="rId63" xr:uid="{86B04D21-DBD4-4B4C-9870-4CCB41BE6157}"/>
-    <hyperlink ref="B69" r:id="rId64" xr:uid="{14150122-3177-4ABC-ACD9-B0B0497B02C1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId65"/>
+  <pageSetup orientation="portrait" r:id="rId64"/>
 </worksheet>
 </file>
</xml_diff>